<commit_message>
Feature: implementação da funcionalidade de enviar email especifico para cada setor
</commit_message>
<xml_diff>
--- a/data/saida/relatorio_vendas.xlsx
+++ b/data/saida/relatorio_vendas.xlsx
@@ -10,8 +10,9 @@
     <sheet name="Resumo" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="Mensal" sheetId="2" state="visible" r:id="rId2"/>
     <sheet name="Categorias" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Produtos" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="Vendedores" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="Produtos (Faturamento)" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Produtos (Quantidade)" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="Vendedores" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -420,7 +421,7 @@
           <order val="0"/>
           <tx>
             <strRef>
-              <f>'Produtos'!B1</f>
+              <f>'Produtos (Faturamento)'!B1</f>
             </strRef>
           </tx>
           <spPr>
@@ -433,12 +434,12 @@
           </spPr>
           <cat>
             <numRef>
-              <f>'Produtos'!$A$2:$A$30</f>
+              <f>'Produtos (Faturamento)'!$A$2:$A$30</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'Produtos'!$B$2:$B$30</f>
+              <f>'Produtos (Faturamento)'!$B$2:$B$30</f>
             </numRef>
           </val>
         </ser>
@@ -513,6 +514,127 @@
 </file>
 
 <file path=xl/charts/chart4.xml><?xml version="1.0" encoding="utf-8"?>
+<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+  <chart>
+    <title>
+      <tx>
+        <rich>
+          <a:bodyPr/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr/>
+            </a:pPr>
+            <a:r>
+              <a:t>Quantidade por Produto</a:t>
+            </a:r>
+          </a:p>
+        </rich>
+      </tx>
+      <overlay val="0"/>
+    </title>
+    <plotArea>
+      <barChart>
+        <barDir val="bar"/>
+        <grouping val="clustered"/>
+        <varyColors val="0"/>
+        <ser>
+          <idx val="0"/>
+          <order val="0"/>
+          <tx>
+            <strRef>
+              <f>'Produtos (Quantidade)'!B1</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:solidFill>
+              <a:srgbClr val="1F4E78"/>
+            </a:solidFill>
+            <a:ln>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <cat>
+            <numRef>
+              <f>'Produtos (Quantidade)'!$A$2:$A$30</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'Produtos (Quantidade)'!$B$2:$B$30</f>
+            </numRef>
+          </val>
+        </ser>
+        <gapWidth val="150"/>
+        <axId val="10"/>
+        <axId val="100"/>
+      </barChart>
+      <catAx>
+        <axId val="10"/>
+        <scaling>
+          <orientation val="maxMin"/>
+        </scaling>
+        <delete val="0"/>
+        <axPos val="l"/>
+        <title>
+          <tx>
+            <rich>
+              <a:bodyPr/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr/>
+                </a:pPr>
+                <a:r>
+                  <a:t>Produto</a:t>
+                </a:r>
+              </a:p>
+            </rich>
+          </tx>
+          <overlay val="0"/>
+        </title>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="100"/>
+        <lblOffset val="100"/>
+        <tickLblSkip val="1"/>
+      </catAx>
+      <valAx>
+        <axId val="100"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <delete val="0"/>
+        <axPos val="l"/>
+        <majorGridlines/>
+        <title>
+          <tx>
+            <rich>
+              <a:bodyPr/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr/>
+                </a:pPr>
+                <a:r>
+                  <a:t>Unidades vendidas</a:t>
+                </a:r>
+              </a:p>
+            </rich>
+          </tx>
+          <overlay val="0"/>
+        </title>
+        <numFmt formatCode="0" sourceLinked="0"/>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="10"/>
+        <crosses val="max"/>
+      </valAx>
+    </plotArea>
+    <plotVisOnly val="1"/>
+    <dispBlanksAs val="gap"/>
+  </chart>
+</chartSpace>
+</file>
+
+<file path=xl/charts/chart5.xml><?xml version="1.0" encoding="utf-8"?>
 <chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <chart>
     <title>
@@ -715,6 +837,33 @@
 </file>
 
 <file path=xl/drawings/drawing4.xml><?xml version="1.0" encoding="utf-8"?>
+<wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+  <oneCellAnchor>
+    <from>
+      <col>3</col>
+      <colOff>0</colOff>
+      <row>1</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="8640000" cy="6263999"/>
+    <graphicFrame>
+      <nvGraphicFramePr>
+        <cNvPr id="1" name="Chart 1"/>
+        <cNvGraphicFramePr/>
+      </nvGraphicFramePr>
+      <xfrm/>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart r:id="rId1"/>
+        </a:graphicData>
+      </a:graphic>
+    </graphicFrame>
+    <clientData/>
+  </oneCellAnchor>
+</wsDr>
+</file>
+
+<file path=xl/drawings/drawing5.xml><?xml version="1.0" encoding="utf-8"?>
 <wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <oneCellAnchor>
     <from>
@@ -1030,7 +1179,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B9"/>
+  <dimension ref="A1:B11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -1116,22 +1265,44 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Melhor vendedor</t>
+          <t>Produto mais vendido</t>
         </is>
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>Maria</t>
+          <t>Mouse Gamer</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
+          <t>Quantidade do produto mais vendido</t>
+        </is>
+      </c>
+      <c r="B9" s="2" t="n">
+        <v>996</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Melhor vendedor</t>
+        </is>
+      </c>
+      <c r="B10" s="2" t="inlineStr">
+        <is>
+          <t>Maria</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
           <t>Faturamento do melhor vendedor</t>
         </is>
       </c>
-      <c r="B9" s="1" t="n">
+      <c r="B11" s="1" t="n">
         <v>4347180</v>
       </c>
     </row>
@@ -1993,6 +2164,327 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:B30"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="28" customWidth="1" min="1" max="1"/>
+    <col width="18" customWidth="1" min="2" max="2"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>Produto</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>unidades</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Mouse Gamer</t>
+        </is>
+      </c>
+      <c r="B2" t="n">
+        <v>996</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Carregador USB-C</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
+        <v>936</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Mouse Ergonômico</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
+        <v>913</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Notebook Básico</t>
+        </is>
+      </c>
+      <c r="B5" t="n">
+        <v>907</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Earbuds</t>
+        </is>
+      </c>
+      <c r="B6" t="n">
+        <v>906</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Mouse Básico</t>
+        </is>
+      </c>
+      <c r="B7" t="n">
+        <v>902</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Headphone Bluetooth</t>
+        </is>
+      </c>
+      <c r="B8" t="n">
+        <v>891</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Smartphone Básico</t>
+        </is>
+      </c>
+      <c r="B9" t="n">
+        <v>889</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Notebook Gamer</t>
+        </is>
+      </c>
+      <c r="B10" t="n">
+        <v>889</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Caixa de Som Bluetooth</t>
+        </is>
+      </c>
+      <c r="B11" t="n">
+        <v>882</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>Smartphone 5G</t>
+        </is>
+      </c>
+      <c r="B12" t="n">
+        <v>875</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>Adaptador USB</t>
+        </is>
+      </c>
+      <c r="B13" t="n">
+        <v>874</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>Teclado de Membrana</t>
+        </is>
+      </c>
+      <c r="B14" t="n">
+        <v>873</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>Smartphone Intermediário</t>
+        </is>
+      </c>
+      <c r="B15" t="n">
+        <v>867</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>Impressora Fotográfica</t>
+        </is>
+      </c>
+      <c r="B16" t="n">
+        <v>866</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>Impressora Jato de Tinta</t>
+        </is>
+      </c>
+      <c r="B17" t="n">
+        <v>865</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>SSD 1TB</t>
+        </is>
+      </c>
+      <c r="B18" t="n">
+        <v>862</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>Cabo USB-C</t>
+        </is>
+      </c>
+      <c r="B19" t="n">
+        <v>859</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>Carregador Sem Fio</t>
+        </is>
+      </c>
+      <c r="B20" t="n">
+        <v>843</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>Headphone Básico</t>
+        </is>
+      </c>
+      <c r="B21" t="n">
+        <v>836</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>HD Externo</t>
+        </is>
+      </c>
+      <c r="B22" t="n">
+        <v>835</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>Pendrive</t>
+        </is>
+      </c>
+      <c r="B23" t="n">
+        <v>820</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>Teclado Sem Fio</t>
+        </is>
+      </c>
+      <c r="B24" t="n">
+        <v>817</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>Headset Gamer</t>
+        </is>
+      </c>
+      <c r="B25" t="n">
+        <v>815</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>Impressora Laser</t>
+        </is>
+      </c>
+      <c r="B26" t="n">
+        <v>813</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>Notebook Intermediário</t>
+        </is>
+      </c>
+      <c r="B27" t="n">
+        <v>794</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>Smartphone Avançado</t>
+        </is>
+      </c>
+      <c r="B28" t="n">
+        <v>789</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>Impressora Multifuncional</t>
+        </is>
+      </c>
+      <c r="B29" t="n">
+        <v>789</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>Teclado Mecânico</t>
+        </is>
+      </c>
+      <c r="B30" t="n">
+        <v>774</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:B7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>

</xml_diff>